<commit_message>
Canvi nom a sankey (bug fix)
</commit_message>
<xml_diff>
--- a/data/punts/punts-mesura-at.xlsx
+++ b/data/punts/punts-mesura-at.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\punts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B0754F07-5958-419A-84EE-617DD9643AE7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFDC6187-A128-43B5-BBC5-A1100F6C7CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -805,7 +805,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -814,9 +814,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
@@ -1177,10 +1174,10 @@
     <col min="5" max="5" width="10.77734375" style="1" customWidth="1"/>
     <col min="6" max="6" width="11.44140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="8.88671875" style="1"/>
-    <col min="8" max="9" width="9.5546875" style="7" customWidth="1"/>
+    <col min="8" max="9" width="9.5546875" style="6" customWidth="1"/>
     <col min="10" max="10" width="11" style="1" customWidth="1"/>
     <col min="11" max="11" width="13.109375" style="1" customWidth="1"/>
-    <col min="12" max="12" width="17.109375" style="7" customWidth="1"/>
+    <col min="12" max="12" width="17.109375" style="6" customWidth="1"/>
     <col min="13" max="13" width="21.44140625" style="1" customWidth="1"/>
     <col min="14" max="14" width="21.77734375" style="1" customWidth="1"/>
     <col min="15" max="16384" width="8.88671875" style="1"/>
@@ -1208,10 +1205,10 @@
       <c r="G1" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="5" t="s">
+      <c r="H1" s="4" t="s">
         <v>86</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>87</v>
       </c>
       <c r="J1" s="2" t="s">
@@ -1220,7 +1217,7 @@
       <c r="K1" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="L1" s="5" t="s">
+      <c r="L1" s="4" t="s">
         <v>88</v>
       </c>
       <c r="M1" s="2" t="s">
@@ -1252,29 +1249,29 @@
       <c r="G2" s="3">
         <v>150</v>
       </c>
-      <c r="H2" s="6">
+      <c r="H2" s="5">
         <v>168.3</v>
       </c>
-      <c r="I2" s="6">
+      <c r="I2" s="5">
         <v>4.8</v>
       </c>
       <c r="J2" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K2" s="4">
-        <f>PI()*(((H2-I2)*10^-3)^2/4)</f>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L2" s="6">
+      <c r="K2" s="3">
+        <f>PI()*(((H2-2*I2)*10^-3)^2/4)</f>
+        <v>1.9780794669897482E-2</v>
+      </c>
+      <c r="L2" s="5">
         <v>3</v>
       </c>
-      <c r="M2" s="4">
-        <f>L2*K2</f>
-        <v>6.2986380160444319E-2</v>
-      </c>
-      <c r="N2" s="4">
+      <c r="M2" s="3">
+        <f t="shared" ref="M2:M33" si="0">L2*K2</f>
+        <v>5.9342384009692446E-2</v>
+      </c>
+      <c r="N2" s="3">
         <f>M2*3600</f>
-        <v>226.75096857759954</v>
+        <v>213.63258243489281</v>
       </c>
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.3">
@@ -1299,29 +1296,29 @@
       <c r="G3" s="3">
         <v>150</v>
       </c>
-      <c r="H3" s="6">
+      <c r="H3" s="5">
         <v>168.3</v>
       </c>
-      <c r="I3" s="6">
+      <c r="I3" s="5">
         <v>4.8</v>
       </c>
       <c r="J3" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K3" s="4">
-        <f>PI()*(((H3-I3)*10^-3)^2/4)</f>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L3" s="6">
+      <c r="K3" s="3">
+        <f t="shared" ref="K3:K66" si="1">PI()*(((H3-2*I3)*10^-3)^2/4)</f>
+        <v>1.9780794669897482E-2</v>
+      </c>
+      <c r="L3" s="5">
         <v>3</v>
       </c>
-      <c r="M3" s="4">
-        <f>L3*K3</f>
-        <v>6.2986380160444319E-2</v>
-      </c>
-      <c r="N3" s="4">
-        <f t="shared" ref="N3:N66" si="0">M3*3600</f>
-        <v>226.75096857759954</v>
+      <c r="M3" s="3">
+        <f t="shared" si="0"/>
+        <v>5.9342384009692446E-2</v>
+      </c>
+      <c r="N3" s="3">
+        <f t="shared" ref="N3:N66" si="2">M3*3600</f>
+        <v>213.63258243489281</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
@@ -1346,29 +1343,29 @@
       <c r="G4" s="3">
         <v>150</v>
       </c>
-      <c r="H4" s="6">
+      <c r="H4" s="5">
         <v>168.3</v>
       </c>
-      <c r="I4" s="6">
+      <c r="I4" s="5">
         <v>4.8</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K4" s="4">
-        <f t="shared" ref="K3:K33" si="1">PI()*(((H4-I4)*10^-3)^2/4)</f>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L4" s="6">
+      <c r="K4" s="3">
+        <f t="shared" si="1"/>
+        <v>1.9780794669897482E-2</v>
+      </c>
+      <c r="L4" s="5">
         <v>3</v>
       </c>
-      <c r="M4" s="4">
-        <f>L4*K4</f>
-        <v>6.2986380160444319E-2</v>
-      </c>
-      <c r="N4" s="4">
+      <c r="M4" s="3">
         <f t="shared" si="0"/>
-        <v>226.75096857759954</v>
+        <v>5.9342384009692446E-2</v>
+      </c>
+      <c r="N4" s="3">
+        <f t="shared" si="2"/>
+        <v>213.63258243489281</v>
       </c>
     </row>
     <row r="5" spans="1:14" x14ac:dyDescent="0.3">
@@ -1393,29 +1390,29 @@
       <c r="G5" s="3">
         <v>150</v>
       </c>
-      <c r="H5" s="6">
+      <c r="H5" s="5">
         <v>168.3</v>
       </c>
-      <c r="I5" s="6">
+      <c r="I5" s="5">
         <v>4.8</v>
       </c>
       <c r="J5" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K5" s="4">
-        <f t="shared" si="1"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L5" s="6">
+      <c r="K5" s="3">
+        <f t="shared" si="1"/>
+        <v>1.9780794669897482E-2</v>
+      </c>
+      <c r="L5" s="5">
         <v>3.4</v>
       </c>
-      <c r="M5" s="4">
-        <f>L5*K5</f>
-        <v>7.138456418183689E-2</v>
-      </c>
-      <c r="N5" s="4">
+      <c r="M5" s="3">
         <f t="shared" si="0"/>
-        <v>256.9844310546128</v>
+        <v>6.7254701877651438E-2</v>
+      </c>
+      <c r="N5" s="3">
+        <f t="shared" si="2"/>
+        <v>242.11692675954518</v>
       </c>
     </row>
     <row r="6" spans="1:14" x14ac:dyDescent="0.3">
@@ -1440,29 +1437,29 @@
       <c r="G6" s="3">
         <v>150</v>
       </c>
-      <c r="H6" s="6">
+      <c r="H6" s="5">
         <v>168.3</v>
       </c>
-      <c r="I6" s="6">
+      <c r="I6" s="5">
         <v>4.8</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K6" s="4">
-        <f t="shared" si="1"/>
-        <v>2.0995460053481439E-2</v>
-      </c>
-      <c r="L6" s="6">
+      <c r="K6" s="3">
+        <f t="shared" si="1"/>
+        <v>1.9780794669897482E-2</v>
+      </c>
+      <c r="L6" s="5">
         <v>3.4</v>
       </c>
-      <c r="M6" s="4">
-        <f>L6*K6</f>
-        <v>7.138456418183689E-2</v>
-      </c>
-      <c r="N6" s="4">
+      <c r="M6" s="3">
         <f t="shared" si="0"/>
-        <v>256.9844310546128</v>
+        <v>6.7254701877651438E-2</v>
+      </c>
+      <c r="N6" s="3">
+        <f t="shared" si="2"/>
+        <v>242.11692675954518</v>
       </c>
     </row>
     <row r="7" spans="1:14" x14ac:dyDescent="0.3">
@@ -1487,29 +1484,29 @@
       <c r="G7" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="H7" s="6">
+      <c r="H7" s="5">
         <v>204</v>
       </c>
-      <c r="I7" s="6">
+      <c r="I7" s="5">
         <v>4.8</v>
       </c>
       <c r="J7" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K7" s="4">
-        <f t="shared" si="1"/>
-        <v>3.116510177843532E-2</v>
-      </c>
-      <c r="L7" s="6">
+      <c r="K7" s="3">
+        <f t="shared" si="1"/>
+        <v>2.9681264736291797E-2</v>
+      </c>
+      <c r="L7" s="5">
         <v>1.35</v>
       </c>
-      <c r="M7" s="4">
-        <f>L7*K7</f>
-        <v>4.2072887400887687E-2</v>
-      </c>
-      <c r="N7" s="4">
+      <c r="M7" s="3">
         <f t="shared" si="0"/>
-        <v>151.46239464319567</v>
+        <v>4.0069707393993931E-2</v>
+      </c>
+      <c r="N7" s="3">
+        <f t="shared" si="2"/>
+        <v>144.25094661837815</v>
       </c>
     </row>
     <row r="8" spans="1:14" x14ac:dyDescent="0.3">
@@ -1534,29 +1531,29 @@
       <c r="G8" s="3">
         <v>350</v>
       </c>
-      <c r="H8" s="6">
+      <c r="H8" s="5">
         <v>355.6</v>
       </c>
-      <c r="I8" s="6">
+      <c r="I8" s="5">
         <v>8</v>
       </c>
       <c r="J8" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K8" s="4">
-        <f t="shared" si="1"/>
-        <v>9.4896329995100878E-2</v>
-      </c>
-      <c r="L8" s="6">
+      <c r="K8" s="3">
+        <f t="shared" si="1"/>
+        <v>9.0578525052007072E-2</v>
+      </c>
+      <c r="L8" s="5">
         <v>2.35</v>
       </c>
-      <c r="M8" s="4">
-        <f>L8*K8</f>
-        <v>0.22300637548848706</v>
-      </c>
-      <c r="N8" s="4">
+      <c r="M8" s="3">
         <f t="shared" si="0"/>
-        <v>802.82295175855347</v>
+        <v>0.21285953387221662</v>
+      </c>
+      <c r="N8" s="3">
+        <f t="shared" si="2"/>
+        <v>766.2943219399798</v>
       </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.3">
@@ -1581,24 +1578,24 @@
       <c r="G9" s="3">
         <v>200</v>
       </c>
-      <c r="H9" s="6">
+      <c r="H9" s="5">
         <v>220</v>
       </c>
-      <c r="I9" s="6"/>
+      <c r="I9" s="5"/>
       <c r="J9" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K9" s="4">
+      <c r="K9" s="3">
         <f t="shared" si="1"/>
         <v>3.8013271108436497E-2</v>
       </c>
-      <c r="L9" s="6"/>
-      <c r="M9" s="4">
-        <f>L9*K9</f>
-        <v>0</v>
-      </c>
-      <c r="N9" s="4">
+      <c r="L9" s="5"/>
+      <c r="M9" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N9" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1624,26 +1621,26 @@
       <c r="G10" s="3">
         <v>80</v>
       </c>
-      <c r="H10" s="6">
+      <c r="H10" s="5">
         <v>88.9</v>
       </c>
-      <c r="I10" s="6">
+      <c r="I10" s="5">
         <v>4</v>
       </c>
       <c r="J10" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K10" s="4">
-        <f t="shared" si="1"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L10" s="6"/>
-      <c r="M10" s="4">
-        <f>L10*K10</f>
-        <v>0</v>
-      </c>
-      <c r="N10" s="4">
+      <c r="K10" s="3">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L10" s="5"/>
+      <c r="M10" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N10" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1669,26 +1666,26 @@
       <c r="G11" s="3">
         <v>80</v>
       </c>
-      <c r="H11" s="6">
+      <c r="H11" s="5">
         <v>88.9</v>
       </c>
-      <c r="I11" s="6">
+      <c r="I11" s="5">
         <v>4</v>
       </c>
       <c r="J11" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K11" s="4">
-        <f t="shared" si="1"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L11" s="6"/>
-      <c r="M11" s="4">
-        <f>L11*K11</f>
-        <v>0</v>
-      </c>
-      <c r="N11" s="4">
+      <c r="K11" s="3">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L11" s="5"/>
+      <c r="M11" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N11" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1714,26 +1711,26 @@
       <c r="G12" s="3">
         <v>65</v>
       </c>
-      <c r="H12" s="6">
+      <c r="H12" s="5">
         <v>76.099999999999994</v>
       </c>
-      <c r="I12" s="6">
+      <c r="I12" s="5">
         <v>3.6</v>
       </c>
       <c r="J12" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K12" s="4">
-        <f t="shared" si="1"/>
-        <v>4.1282490963578371E-3</v>
-      </c>
-      <c r="L12" s="6"/>
-      <c r="M12" s="4">
-        <f>L12*K12</f>
-        <v>0</v>
-      </c>
-      <c r="N12" s="4">
+      <c r="K12" s="3">
+        <f t="shared" si="1"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L12" s="5"/>
+      <c r="M12" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N12" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1759,26 +1756,26 @@
       <c r="G13" s="3">
         <v>100</v>
       </c>
-      <c r="H13" s="6">
+      <c r="H13" s="5">
         <v>114</v>
       </c>
-      <c r="I13" s="6">
+      <c r="I13" s="5">
         <v>4.5</v>
       </c>
       <c r="J13" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K13" s="4">
-        <f t="shared" si="1"/>
-        <v>9.4171203286762539E-3</v>
-      </c>
-      <c r="L13" s="6"/>
-      <c r="M13" s="4">
-        <f>L13*K13</f>
-        <v>0</v>
-      </c>
-      <c r="N13" s="4">
+      <c r="K13" s="3">
+        <f t="shared" si="1"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="L13" s="5"/>
+      <c r="M13" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N13" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1802,22 +1799,22 @@
         <v>33</v>
       </c>
       <c r="G14" s="3"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
+      <c r="H14" s="5"/>
+      <c r="I14" s="5"/>
       <c r="J14" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K14" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L14" s="6"/>
-      <c r="M14" s="4">
-        <f>L14*K14</f>
-        <v>0</v>
-      </c>
-      <c r="N14" s="4">
+      <c r="K14" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L14" s="5"/>
+      <c r="M14" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N14" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1841,22 +1838,22 @@
         <v>34</v>
       </c>
       <c r="G15" s="3"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
+      <c r="H15" s="5"/>
+      <c r="I15" s="5"/>
       <c r="J15" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K15" s="4">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="L15" s="6"/>
-      <c r="M15" s="4">
-        <f>L15*K15</f>
-        <v>0</v>
-      </c>
-      <c r="N15" s="4">
+      <c r="K15" s="3">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="L15" s="5"/>
+      <c r="M15" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N15" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1882,26 +1879,26 @@
       <c r="G16" s="3">
         <v>125</v>
       </c>
-      <c r="H16" s="6">
+      <c r="H16" s="5">
         <v>141</v>
       </c>
-      <c r="I16" s="6">
+      <c r="I16" s="5">
         <v>5</v>
       </c>
       <c r="J16" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K16" s="4">
-        <f t="shared" si="1"/>
-        <v>1.4526724430199206E-2</v>
-      </c>
-      <c r="L16" s="6"/>
-      <c r="M16" s="4">
-        <f>L16*K16</f>
-        <v>0</v>
-      </c>
-      <c r="N16" s="4">
+      <c r="K16" s="3">
+        <f t="shared" si="1"/>
+        <v>1.3478217882063612E-2</v>
+      </c>
+      <c r="L16" s="5"/>
+      <c r="M16" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N16" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -1927,29 +1924,29 @@
       <c r="G17" s="3">
         <v>155</v>
       </c>
-      <c r="H17" s="6">
+      <c r="H17" s="5">
         <v>155</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="5">
         <v>1.8</v>
       </c>
       <c r="J17" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K17" s="4">
-        <f t="shared" si="1"/>
-        <v>1.8433483390497326E-2</v>
-      </c>
-      <c r="L17" s="6">
+      <c r="K17" s="3">
+        <f t="shared" si="1"/>
+        <v>1.8002865285469776E-2</v>
+      </c>
+      <c r="L17" s="5">
         <v>0.7</v>
       </c>
-      <c r="M17" s="4">
-        <f>L17*K17</f>
-        <v>1.2903438373348128E-2</v>
-      </c>
-      <c r="N17" s="4">
+      <c r="M17" s="3">
         <f t="shared" si="0"/>
-        <v>46.452378144053263</v>
+        <v>1.2602005699828842E-2</v>
+      </c>
+      <c r="N17" s="3">
+        <f t="shared" si="2"/>
+        <v>45.367220519383828</v>
       </c>
     </row>
     <row r="18" spans="1:14" x14ac:dyDescent="0.3">
@@ -1974,29 +1971,29 @@
       <c r="G18" s="3">
         <v>80</v>
       </c>
-      <c r="H18" s="6">
+      <c r="H18" s="5">
         <v>88.9</v>
       </c>
-      <c r="I18" s="6">
+      <c r="I18" s="5">
         <v>2</v>
       </c>
       <c r="J18" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K18" s="4">
-        <f t="shared" si="1"/>
-        <v>5.9310206246938049E-3</v>
-      </c>
-      <c r="L18" s="6">
+      <c r="K18" s="3">
+        <f t="shared" si="1"/>
+        <v>5.661157815750442E-3</v>
+      </c>
+      <c r="L18" s="5">
         <v>0.5</v>
       </c>
-      <c r="M18" s="4">
-        <f>L18*K18</f>
-        <v>2.9655103123469024E-3</v>
-      </c>
-      <c r="N18" s="4">
+      <c r="M18" s="3">
         <f t="shared" si="0"/>
-        <v>10.675837124448849</v>
+        <v>2.830578907875221E-3</v>
+      </c>
+      <c r="N18" s="3">
+        <f t="shared" si="2"/>
+        <v>10.190084068350796</v>
       </c>
     </row>
     <row r="19" spans="1:14" x14ac:dyDescent="0.3">
@@ -2021,29 +2018,29 @@
       <c r="G19" s="3">
         <v>125</v>
       </c>
-      <c r="H19" s="6">
+      <c r="H19" s="5">
         <v>139.69999999999999</v>
       </c>
-      <c r="I19" s="6">
+      <c r="I19" s="5">
         <v>2</v>
       </c>
       <c r="J19" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K19" s="4">
-        <f t="shared" si="1"/>
-        <v>1.4892162341646401E-2</v>
-      </c>
-      <c r="L19" s="6">
+      <c r="K19" s="3">
+        <f t="shared" si="1"/>
+        <v>1.4462706625900674E-2</v>
+      </c>
+      <c r="L19" s="5">
         <v>0.62</v>
       </c>
-      <c r="M19" s="4">
-        <f>L19*K19</f>
-        <v>9.2331406518207683E-3</v>
-      </c>
-      <c r="N19" s="4">
+      <c r="M19" s="3">
         <f t="shared" si="0"/>
-        <v>33.239306346554763</v>
+        <v>8.9668781080584174E-3</v>
+      </c>
+      <c r="N19" s="3">
+        <f t="shared" si="2"/>
+        <v>32.280761189010306</v>
       </c>
     </row>
     <row r="20" spans="1:14" x14ac:dyDescent="0.3">
@@ -2068,26 +2065,26 @@
       <c r="G20" s="3">
         <v>80</v>
       </c>
-      <c r="H20" s="6">
+      <c r="H20" s="5">
         <v>88.9</v>
       </c>
-      <c r="I20" s="6">
+      <c r="I20" s="5">
         <v>2</v>
       </c>
       <c r="J20" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K20" s="4">
-        <f t="shared" si="1"/>
-        <v>5.9310206246938049E-3</v>
-      </c>
-      <c r="L20" s="6"/>
-      <c r="M20" s="4">
-        <f>L20*K20</f>
-        <v>0</v>
-      </c>
-      <c r="N20" s="4">
+      <c r="K20" s="3">
+        <f t="shared" si="1"/>
+        <v>5.661157815750442E-3</v>
+      </c>
+      <c r="L20" s="5"/>
+      <c r="M20" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N20" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2113,29 +2110,29 @@
       <c r="G21" s="3">
         <v>125</v>
       </c>
-      <c r="H21" s="6">
+      <c r="H21" s="5">
         <v>139.69999999999999</v>
       </c>
-      <c r="I21" s="6">
+      <c r="I21" s="5">
         <v>2</v>
       </c>
       <c r="J21" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K21" s="4">
-        <f t="shared" si="1"/>
-        <v>1.4892162341646401E-2</v>
-      </c>
-      <c r="L21" s="6">
+      <c r="K21" s="3">
+        <f t="shared" si="1"/>
+        <v>1.4462706625900674E-2</v>
+      </c>
+      <c r="L21" s="5">
         <v>0.9</v>
       </c>
-      <c r="M21" s="4">
-        <f>L21*K21</f>
-        <v>1.340294610748176E-2</v>
-      </c>
-      <c r="N21" s="4">
+      <c r="M21" s="3">
         <f t="shared" si="0"/>
-        <v>48.250605986934339</v>
+        <v>1.3016435963310606E-2</v>
+      </c>
+      <c r="N21" s="3">
+        <f t="shared" si="2"/>
+        <v>46.859169467918186</v>
       </c>
     </row>
     <row r="22" spans="1:14" x14ac:dyDescent="0.3">
@@ -2160,26 +2157,26 @@
       <c r="G22" s="3">
         <v>204</v>
       </c>
-      <c r="H22" s="6">
+      <c r="H22" s="5">
         <v>204</v>
       </c>
-      <c r="I22" s="6">
+      <c r="I22" s="5">
         <v>2</v>
       </c>
       <c r="J22" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K22" s="4">
-        <f t="shared" si="1"/>
-        <v>3.2047386659269483E-2</v>
-      </c>
-      <c r="L22" s="6"/>
-      <c r="M22" s="4">
-        <f>L22*K22</f>
-        <v>0</v>
-      </c>
-      <c r="N22" s="4">
+      <c r="K22" s="3">
+        <f t="shared" si="1"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="L22" s="5"/>
+      <c r="M22" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N22" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2205,29 +2202,29 @@
       <c r="G23" s="3">
         <v>204</v>
       </c>
-      <c r="H23" s="6">
+      <c r="H23" s="5">
         <v>204</v>
       </c>
-      <c r="I23" s="6">
+      <c r="I23" s="5">
         <v>2</v>
       </c>
       <c r="J23" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K23" s="4">
-        <f t="shared" si="1"/>
-        <v>3.2047386659269483E-2</v>
-      </c>
-      <c r="L23" s="6">
+      <c r="K23" s="3">
+        <f t="shared" si="1"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="L23" s="5">
         <v>2</v>
       </c>
-      <c r="M23" s="4">
-        <f>L23*K23</f>
-        <v>6.4094773318538967E-2</v>
-      </c>
-      <c r="N23" s="4">
+      <c r="M23" s="3">
         <f t="shared" si="0"/>
-        <v>230.74118394674028</v>
+        <v>6.2831853071795868E-2</v>
+      </c>
+      <c r="N23" s="3">
+        <f t="shared" si="2"/>
+        <v>226.19467105846513</v>
       </c>
     </row>
     <row r="24" spans="1:14" x14ac:dyDescent="0.3">
@@ -2252,26 +2249,26 @@
       <c r="G24" s="3">
         <v>80</v>
       </c>
-      <c r="H24" s="6">
+      <c r="H24" s="5">
         <v>88.9</v>
       </c>
-      <c r="I24" s="6">
+      <c r="I24" s="5">
         <v>2</v>
       </c>
       <c r="J24" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K24" s="4">
-        <f t="shared" si="1"/>
-        <v>5.9310206246938049E-3</v>
-      </c>
-      <c r="L24" s="6"/>
-      <c r="M24" s="4">
-        <f>L24*K24</f>
-        <v>0</v>
-      </c>
-      <c r="N24" s="4">
+      <c r="K24" s="3">
+        <f t="shared" si="1"/>
+        <v>5.661157815750442E-3</v>
+      </c>
+      <c r="L24" s="5"/>
+      <c r="M24" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N24" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2297,29 +2294,29 @@
       <c r="G25" s="3">
         <v>125</v>
       </c>
-      <c r="H25" s="6">
+      <c r="H25" s="5">
         <v>139.69999999999999</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="5">
         <v>2</v>
       </c>
       <c r="J25" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K25" s="4">
-        <f t="shared" si="1"/>
-        <v>1.4892162341646401E-2</v>
-      </c>
-      <c r="L25" s="6">
+      <c r="K25" s="3">
+        <f t="shared" si="1"/>
+        <v>1.4462706625900674E-2</v>
+      </c>
+      <c r="L25" s="5">
         <v>1.8</v>
       </c>
-      <c r="M25" s="4">
-        <f>L25*K25</f>
-        <v>2.6805892214963521E-2</v>
-      </c>
-      <c r="N25" s="4">
+      <c r="M25" s="3">
         <f t="shared" si="0"/>
-        <v>96.501211973868678</v>
+        <v>2.6032871926621213E-2</v>
+      </c>
+      <c r="N25" s="3">
+        <f t="shared" si="2"/>
+        <v>93.718338935836371</v>
       </c>
     </row>
     <row r="26" spans="1:14" x14ac:dyDescent="0.3">
@@ -2344,29 +2341,29 @@
       <c r="G26" s="3">
         <v>155</v>
       </c>
-      <c r="H26" s="6">
+      <c r="H26" s="5">
         <v>154</v>
       </c>
-      <c r="I26" s="6">
+      <c r="I26" s="5">
         <v>2</v>
       </c>
       <c r="J26" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K26" s="4">
-        <f t="shared" si="1"/>
-        <v>1.8145839167134643E-2</v>
-      </c>
-      <c r="L26" s="6">
+      <c r="K26" s="3">
+        <f t="shared" si="1"/>
+        <v>1.7671458676442587E-2</v>
+      </c>
+      <c r="L26" s="5">
         <v>2.5</v>
       </c>
-      <c r="M26" s="4">
-        <f>L26*K26</f>
-        <v>4.5364597917836605E-2</v>
-      </c>
-      <c r="N26" s="4">
+      <c r="M26" s="3">
         <f t="shared" si="0"/>
-        <v>163.31255250421177</v>
+        <v>4.4178646691106466E-2</v>
+      </c>
+      <c r="N26" s="3">
+        <f t="shared" si="2"/>
+        <v>159.04312808798326</v>
       </c>
     </row>
     <row r="27" spans="1:14" x14ac:dyDescent="0.3">
@@ -2391,29 +2388,29 @@
       <c r="G27" s="3">
         <v>204</v>
       </c>
-      <c r="H27" s="6">
+      <c r="H27" s="5">
         <v>204</v>
       </c>
-      <c r="I27" s="6">
+      <c r="I27" s="5">
         <v>2</v>
       </c>
       <c r="J27" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K27" s="4">
-        <f t="shared" si="1"/>
-        <v>3.2047386659269483E-2</v>
-      </c>
-      <c r="L27" s="6">
+      <c r="K27" s="3">
+        <f t="shared" si="1"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="L27" s="5">
         <v>1.8</v>
       </c>
-      <c r="M27" s="4">
-        <f>L27*K27</f>
-        <v>5.7685295986685071E-2</v>
-      </c>
-      <c r="N27" s="4">
+      <c r="M27" s="3">
         <f t="shared" si="0"/>
-        <v>207.66706555206625</v>
+        <v>5.6548667764616284E-2</v>
+      </c>
+      <c r="N27" s="3">
+        <f t="shared" si="2"/>
+        <v>203.57520395261861</v>
       </c>
     </row>
     <row r="28" spans="1:14" x14ac:dyDescent="0.3">
@@ -2438,29 +2435,29 @@
       <c r="G28" s="3">
         <v>155</v>
       </c>
-      <c r="H28" s="6">
+      <c r="H28" s="5">
         <v>154</v>
       </c>
-      <c r="I28" s="6">
+      <c r="I28" s="5">
         <v>2</v>
       </c>
       <c r="J28" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K28" s="4">
-        <f t="shared" si="1"/>
-        <v>1.8145839167134643E-2</v>
-      </c>
-      <c r="L28" s="6">
+      <c r="K28" s="3">
+        <f t="shared" si="1"/>
+        <v>1.7671458676442587E-2</v>
+      </c>
+      <c r="L28" s="5">
         <v>2.8</v>
       </c>
-      <c r="M28" s="4">
-        <f>L28*K28</f>
-        <v>5.0808349667976996E-2</v>
-      </c>
-      <c r="N28" s="4">
+      <c r="M28" s="3">
         <f t="shared" si="0"/>
-        <v>182.91005880471718</v>
+        <v>4.9480084294039238E-2</v>
+      </c>
+      <c r="N28" s="3">
+        <f t="shared" si="2"/>
+        <v>178.12830345854127</v>
       </c>
     </row>
     <row r="29" spans="1:14" x14ac:dyDescent="0.3">
@@ -2485,26 +2482,26 @@
       <c r="G29" s="3">
         <v>204</v>
       </c>
-      <c r="H29" s="6">
+      <c r="H29" s="5">
         <v>204</v>
       </c>
-      <c r="I29" s="6">
+      <c r="I29" s="5">
         <v>2</v>
       </c>
       <c r="J29" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K29" s="4">
-        <f t="shared" si="1"/>
-        <v>3.2047386659269483E-2</v>
-      </c>
-      <c r="L29" s="6"/>
-      <c r="M29" s="4">
-        <f>L29*K29</f>
-        <v>0</v>
-      </c>
-      <c r="N29" s="4">
+      <c r="K29" s="3">
+        <f t="shared" si="1"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="L29" s="5"/>
+      <c r="M29" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N29" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2526,26 +2523,26 @@
       <c r="G30" s="3">
         <v>129</v>
       </c>
-      <c r="H30" s="6">
+      <c r="H30" s="5">
         <v>129</v>
       </c>
-      <c r="I30" s="6">
+      <c r="I30" s="5">
         <v>2</v>
       </c>
       <c r="J30" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K30" s="4">
-        <f t="shared" si="1"/>
-        <v>1.2667686977437444E-2</v>
-      </c>
-      <c r="L30" s="6"/>
-      <c r="M30" s="4">
-        <f>L30*K30</f>
-        <v>0</v>
-      </c>
-      <c r="N30" s="4">
+      <c r="K30" s="3">
+        <f t="shared" si="1"/>
+        <v>1.2271846303085129E-2</v>
+      </c>
+      <c r="L30" s="5"/>
+      <c r="M30" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N30" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2571,26 +2568,26 @@
       <c r="G31" s="3">
         <v>129</v>
       </c>
-      <c r="H31" s="6">
+      <c r="H31" s="5">
         <v>129</v>
       </c>
-      <c r="I31" s="6">
+      <c r="I31" s="5">
         <v>2</v>
       </c>
       <c r="J31" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K31" s="4">
-        <f t="shared" si="1"/>
-        <v>1.2667686977437444E-2</v>
-      </c>
-      <c r="L31" s="6"/>
-      <c r="M31" s="4">
-        <f>L31*K31</f>
-        <v>0</v>
-      </c>
-      <c r="N31" s="4">
+      <c r="K31" s="3">
+        <f t="shared" si="1"/>
+        <v>1.2271846303085129E-2</v>
+      </c>
+      <c r="L31" s="5"/>
+      <c r="M31" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N31" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2616,26 +2613,26 @@
       <c r="G32" s="3">
         <v>204</v>
       </c>
-      <c r="H32" s="6">
+      <c r="H32" s="5">
         <v>204</v>
       </c>
-      <c r="I32" s="6">
+      <c r="I32" s="5">
         <v>2</v>
       </c>
       <c r="J32" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K32" s="4">
-        <f t="shared" si="1"/>
-        <v>3.2047386659269483E-2</v>
-      </c>
-      <c r="L32" s="6"/>
-      <c r="M32" s="4">
-        <f>L32*K32</f>
-        <v>0</v>
-      </c>
-      <c r="N32" s="4">
+      <c r="K32" s="3">
+        <f t="shared" si="1"/>
+        <v>3.1415926535897934E-2</v>
+      </c>
+      <c r="L32" s="5"/>
+      <c r="M32" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N32" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2661,26 +2658,26 @@
       <c r="G33" s="3">
         <v>100</v>
       </c>
-      <c r="H33" s="6">
+      <c r="H33" s="5">
         <v>114</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="5">
         <v>2</v>
       </c>
       <c r="J33" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K33" s="4">
-        <f t="shared" si="1"/>
-        <v>9.8520345616575928E-3</v>
-      </c>
-      <c r="L33" s="6"/>
-      <c r="M33" s="4">
-        <f>L33*K33</f>
-        <v>0</v>
-      </c>
-      <c r="N33" s="4">
+      <c r="K33" s="3">
+        <f t="shared" si="1"/>
+        <v>9.5033177771091243E-3</v>
+      </c>
+      <c r="L33" s="5"/>
+      <c r="M33" s="3">
         <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="N33" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2706,26 +2703,26 @@
       <c r="G34" s="3">
         <v>65</v>
       </c>
-      <c r="H34" s="6">
+      <c r="H34" s="5">
         <v>76.099999999999994</v>
       </c>
-      <c r="I34" s="6">
+      <c r="I34" s="5">
         <v>3.6</v>
       </c>
       <c r="J34" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K34" s="4">
-        <f t="shared" ref="K34:K65" si="2">PI()*(((H34-I34)*10^-3)^2/4)</f>
-        <v>4.1282490963578371E-3</v>
-      </c>
-      <c r="L34" s="6"/>
-      <c r="M34" s="4">
-        <f>L34*K34</f>
-        <v>0</v>
-      </c>
-      <c r="N34" s="4">
-        <f t="shared" si="0"/>
+      <c r="K34" s="3">
+        <f t="shared" si="1"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L34" s="5"/>
+      <c r="M34" s="3">
+        <f t="shared" ref="M34:M65" si="3">L34*K34</f>
+        <v>0</v>
+      </c>
+      <c r="N34" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2751,26 +2748,26 @@
       <c r="G35" s="3">
         <v>125</v>
       </c>
-      <c r="H35" s="6">
+      <c r="H35" s="5">
         <v>139</v>
       </c>
-      <c r="I35" s="6">
+      <c r="I35" s="5">
         <v>5</v>
       </c>
       <c r="J35" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K35" s="4">
-        <f t="shared" si="2"/>
-        <v>1.4102609421964583E-2</v>
-      </c>
-      <c r="L35" s="6"/>
-      <c r="M35" s="4">
-        <f>L35*K35</f>
-        <v>0</v>
-      </c>
-      <c r="N35" s="4">
-        <f t="shared" si="0"/>
+      <c r="K35" s="3">
+        <f t="shared" si="1"/>
+        <v>1.3069810837096936E-2</v>
+      </c>
+      <c r="L35" s="5"/>
+      <c r="M35" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N35" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2796,26 +2793,26 @@
       <c r="G36" s="3">
         <v>43</v>
       </c>
-      <c r="H36" s="6">
+      <c r="H36" s="5">
         <v>43</v>
       </c>
-      <c r="I36" s="6">
+      <c r="I36" s="5">
         <v>2</v>
       </c>
       <c r="J36" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K36" s="4">
-        <f t="shared" si="2"/>
-        <v>1.3202543126711107E-3</v>
-      </c>
-      <c r="L36" s="6"/>
-      <c r="M36" s="4">
-        <f>L36*K36</f>
-        <v>0</v>
-      </c>
-      <c r="N36" s="4">
-        <f t="shared" si="0"/>
+      <c r="K36" s="3">
+        <f t="shared" si="1"/>
+        <v>1.1945906065275189E-3</v>
+      </c>
+      <c r="L36" s="5"/>
+      <c r="M36" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N36" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2841,26 +2838,26 @@
       <c r="G37" s="3">
         <v>50</v>
       </c>
-      <c r="H37" s="6">
+      <c r="H37" s="5">
         <v>60.3</v>
       </c>
-      <c r="I37" s="6">
+      <c r="I37" s="5">
         <v>3.6</v>
       </c>
       <c r="J37" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K37" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L37" s="6"/>
-      <c r="M37" s="4">
-        <f>L37*K37</f>
-        <v>0</v>
-      </c>
-      <c r="N37" s="4">
-        <f t="shared" si="0"/>
+      <c r="K37" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L37" s="5"/>
+      <c r="M37" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N37" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2886,26 +2883,26 @@
       <c r="G38" s="3">
         <v>50</v>
       </c>
-      <c r="H38" s="6">
+      <c r="H38" s="5">
         <v>60.3</v>
       </c>
-      <c r="I38" s="6">
+      <c r="I38" s="5">
         <v>3.6</v>
       </c>
       <c r="J38" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K38" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L38" s="6"/>
-      <c r="M38" s="4">
-        <f>L38*K38</f>
-        <v>0</v>
-      </c>
-      <c r="N38" s="4">
-        <f t="shared" si="0"/>
+      <c r="K38" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L38" s="5"/>
+      <c r="M38" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N38" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2931,26 +2928,26 @@
       <c r="G39" s="3">
         <v>100</v>
       </c>
-      <c r="H39" s="6">
+      <c r="H39" s="5">
         <v>114</v>
       </c>
-      <c r="I39" s="6">
+      <c r="I39" s="5">
         <v>4.5</v>
       </c>
       <c r="J39" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K39" s="4">
-        <f t="shared" si="2"/>
-        <v>9.4171203286762539E-3</v>
-      </c>
-      <c r="L39" s="6"/>
-      <c r="M39" s="4">
-        <f>L39*K39</f>
-        <v>0</v>
-      </c>
-      <c r="N39" s="4">
-        <f t="shared" si="0"/>
+      <c r="K39" s="3">
+        <f t="shared" si="1"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="L39" s="5"/>
+      <c r="M39" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N39" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -2976,26 +2973,26 @@
       <c r="G40" s="3">
         <v>80</v>
       </c>
-      <c r="H40" s="6">
+      <c r="H40" s="5">
         <v>88.9</v>
       </c>
-      <c r="I40" s="6">
+      <c r="I40" s="5">
         <v>4</v>
       </c>
       <c r="J40" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K40" s="4">
-        <f t="shared" si="2"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L40" s="6"/>
-      <c r="M40" s="4">
-        <f>L40*K40</f>
-        <v>0</v>
-      </c>
-      <c r="N40" s="4">
-        <f t="shared" si="0"/>
+      <c r="K40" s="3">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L40" s="5"/>
+      <c r="M40" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N40" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3021,26 +3018,26 @@
       <c r="G41" s="3">
         <v>50</v>
       </c>
-      <c r="H41" s="6">
+      <c r="H41" s="5">
         <v>60.3</v>
       </c>
-      <c r="I41" s="6">
+      <c r="I41" s="5">
         <v>3.6</v>
       </c>
       <c r="J41" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K41" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L41" s="6"/>
-      <c r="M41" s="4">
-        <f>L41*K41</f>
-        <v>0</v>
-      </c>
-      <c r="N41" s="4">
-        <f t="shared" si="0"/>
+      <c r="K41" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L41" s="5"/>
+      <c r="M41" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N41" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3066,26 +3063,26 @@
       <c r="G42" s="3">
         <v>50</v>
       </c>
-      <c r="H42" s="6">
+      <c r="H42" s="5">
         <v>60.3</v>
       </c>
-      <c r="I42" s="6">
+      <c r="I42" s="5">
         <v>3.6</v>
       </c>
       <c r="J42" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K42" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L42" s="6"/>
-      <c r="M42" s="4">
-        <f>L42*K42</f>
-        <v>0</v>
-      </c>
-      <c r="N42" s="4">
-        <f t="shared" si="0"/>
+      <c r="K42" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L42" s="5"/>
+      <c r="M42" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N42" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3111,26 +3108,26 @@
       <c r="G43" s="3">
         <v>40</v>
       </c>
-      <c r="H43" s="6">
+      <c r="H43" s="5">
         <v>48.3</v>
       </c>
-      <c r="I43" s="6">
+      <c r="I43" s="5">
         <v>3.2</v>
       </c>
       <c r="J43" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K43" s="4">
-        <f t="shared" si="2"/>
-        <v>1.5975077183320431E-3</v>
-      </c>
-      <c r="L43" s="6"/>
-      <c r="M43" s="4">
-        <f>L43*K43</f>
-        <v>0</v>
-      </c>
-      <c r="N43" s="4">
-        <f t="shared" si="0"/>
+      <c r="K43" s="3">
+        <f t="shared" si="1"/>
+        <v>1.378852869642194E-3</v>
+      </c>
+      <c r="L43" s="5"/>
+      <c r="M43" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N43" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3156,26 +3153,26 @@
       <c r="G44" s="3">
         <v>40</v>
       </c>
-      <c r="H44" s="6">
+      <c r="H44" s="5">
         <v>48.3</v>
       </c>
-      <c r="I44" s="6">
+      <c r="I44" s="5">
         <v>3.2</v>
       </c>
       <c r="J44" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K44" s="4">
-        <f t="shared" si="2"/>
-        <v>1.5975077183320431E-3</v>
-      </c>
-      <c r="L44" s="6"/>
-      <c r="M44" s="4">
-        <f>L44*K44</f>
-        <v>0</v>
-      </c>
-      <c r="N44" s="4">
-        <f t="shared" si="0"/>
+      <c r="K44" s="3">
+        <f t="shared" si="1"/>
+        <v>1.378852869642194E-3</v>
+      </c>
+      <c r="L44" s="5"/>
+      <c r="M44" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N44" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3201,26 +3198,26 @@
       <c r="G45" s="3">
         <v>50</v>
       </c>
-      <c r="H45" s="6">
+      <c r="H45" s="5">
         <v>60.3</v>
       </c>
-      <c r="I45" s="6">
+      <c r="I45" s="5">
         <v>3.6</v>
       </c>
       <c r="J45" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K45" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L45" s="6"/>
-      <c r="M45" s="4">
-        <f>L45*K45</f>
-        <v>0</v>
-      </c>
-      <c r="N45" s="4">
-        <f t="shared" si="0"/>
+      <c r="K45" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L45" s="5"/>
+      <c r="M45" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N45" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3246,26 +3243,26 @@
       <c r="G46" s="3">
         <v>50</v>
       </c>
-      <c r="H46" s="6">
+      <c r="H46" s="5">
         <v>60.3</v>
       </c>
-      <c r="I46" s="6">
+      <c r="I46" s="5">
         <v>3.6</v>
       </c>
       <c r="J46" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K46" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L46" s="6"/>
-      <c r="M46" s="4">
-        <f>L46*K46</f>
-        <v>0</v>
-      </c>
-      <c r="N46" s="4">
-        <f t="shared" si="0"/>
+      <c r="K46" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L46" s="5"/>
+      <c r="M46" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N46" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3291,26 +3288,26 @@
       <c r="G47" s="3">
         <v>50</v>
       </c>
-      <c r="H47" s="6">
+      <c r="H47" s="5">
         <v>60.3</v>
       </c>
-      <c r="I47" s="6">
+      <c r="I47" s="5">
         <v>3.6</v>
       </c>
       <c r="J47" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K47" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L47" s="6"/>
-      <c r="M47" s="4">
-        <f>L47*K47</f>
-        <v>0</v>
-      </c>
-      <c r="N47" s="4">
-        <f t="shared" si="0"/>
+      <c r="K47" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L47" s="5"/>
+      <c r="M47" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N47" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3336,24 +3333,24 @@
       <c r="G48" s="3">
         <v>200</v>
       </c>
-      <c r="H48" s="6">
+      <c r="H48" s="5">
         <v>220</v>
       </c>
-      <c r="I48" s="6"/>
+      <c r="I48" s="5"/>
       <c r="J48" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K48" s="4">
-        <f t="shared" si="2"/>
+      <c r="K48" s="3">
+        <f t="shared" si="1"/>
         <v>3.8013271108436497E-2</v>
       </c>
-      <c r="L48" s="6"/>
-      <c r="M48" s="4">
-        <f>L48*K48</f>
-        <v>0</v>
-      </c>
-      <c r="N48" s="4">
-        <f t="shared" si="0"/>
+      <c r="L48" s="5"/>
+      <c r="M48" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N48" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3379,26 +3376,26 @@
       <c r="G49" s="3">
         <v>50</v>
       </c>
-      <c r="H49" s="6">
+      <c r="H49" s="5">
         <v>60.3</v>
       </c>
-      <c r="I49" s="6">
+      <c r="I49" s="5">
         <v>3.6</v>
       </c>
       <c r="J49" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K49" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L49" s="6"/>
-      <c r="M49" s="4">
-        <f>L49*K49</f>
-        <v>0</v>
-      </c>
-      <c r="N49" s="4">
-        <f t="shared" si="0"/>
+      <c r="K49" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L49" s="5"/>
+      <c r="M49" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N49" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3424,29 +3421,29 @@
       <c r="G50" s="3">
         <v>125</v>
       </c>
-      <c r="H50" s="6">
+      <c r="H50" s="5">
         <v>141</v>
       </c>
-      <c r="I50" s="6">
+      <c r="I50" s="5">
         <v>5</v>
       </c>
       <c r="J50" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K50" s="4">
-        <f t="shared" si="2"/>
-        <v>1.4526724430199206E-2</v>
-      </c>
-      <c r="L50" s="6">
+      <c r="K50" s="3">
+        <f t="shared" si="1"/>
+        <v>1.3478217882063612E-2</v>
+      </c>
+      <c r="L50" s="5">
         <v>1.9</v>
       </c>
-      <c r="M50" s="4">
-        <f>L50*K50</f>
-        <v>2.760077641737849E-2</v>
-      </c>
-      <c r="N50" s="4">
-        <f t="shared" si="0"/>
-        <v>99.362795102562558</v>
+      <c r="M50" s="3">
+        <f t="shared" si="3"/>
+        <v>2.560861397592086E-2</v>
+      </c>
+      <c r="N50" s="3">
+        <f t="shared" si="2"/>
+        <v>92.191010313315104</v>
       </c>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
@@ -3471,29 +3468,29 @@
       <c r="G51" s="3">
         <v>80</v>
       </c>
-      <c r="H51" s="6">
+      <c r="H51" s="5">
         <v>88.9</v>
       </c>
-      <c r="I51" s="6">
+      <c r="I51" s="5">
         <v>4</v>
       </c>
       <c r="J51" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K51" s="4">
-        <f t="shared" si="2"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L51" s="6">
+      <c r="K51" s="3">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L51" s="5">
         <v>3</v>
       </c>
-      <c r="M51" s="4">
-        <f>L51*K51</f>
-        <v>1.6983473447251325E-2</v>
-      </c>
-      <c r="N51" s="4">
-        <f t="shared" si="0"/>
-        <v>61.140504410104768</v>
+      <c r="M51" s="3">
+        <f t="shared" si="3"/>
+        <v>1.5420845261355766E-2</v>
+      </c>
+      <c r="N51" s="3">
+        <f t="shared" si="2"/>
+        <v>55.515042940880754</v>
       </c>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
@@ -3518,29 +3515,29 @@
       <c r="G52" s="3">
         <v>80</v>
       </c>
-      <c r="H52" s="6">
+      <c r="H52" s="5">
         <v>88.9</v>
       </c>
-      <c r="I52" s="6">
+      <c r="I52" s="5">
         <v>4</v>
       </c>
       <c r="J52" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K52" s="4">
-        <f t="shared" si="2"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L52" s="6">
+      <c r="K52" s="3">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L52" s="5">
         <v>0.46</v>
       </c>
-      <c r="M52" s="4">
-        <f>L52*K52</f>
-        <v>2.6041325952452033E-3</v>
-      </c>
-      <c r="N52" s="4">
-        <f t="shared" si="0"/>
-        <v>9.3748773428827317</v>
+      <c r="M52" s="3">
+        <f t="shared" si="3"/>
+        <v>2.3645296067412178E-3</v>
+      </c>
+      <c r="N52" s="3">
+        <f t="shared" si="2"/>
+        <v>8.5123065842683836</v>
       </c>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
@@ -3565,29 +3562,29 @@
       <c r="G53" s="3">
         <v>50</v>
       </c>
-      <c r="H53" s="6">
+      <c r="H53" s="5">
         <v>60.3</v>
       </c>
-      <c r="I53" s="6">
+      <c r="I53" s="5">
         <v>3.6</v>
       </c>
       <c r="J53" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K53" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L53" s="6">
+      <c r="K53" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L53" s="5">
         <v>3</v>
       </c>
-      <c r="M53" s="4">
-        <f>L53*K53</f>
-        <v>7.5749061045744664E-3</v>
-      </c>
-      <c r="N53" s="4">
-        <f t="shared" si="0"/>
-        <v>27.269661976468079</v>
+      <c r="M53" s="3">
+        <f t="shared" si="3"/>
+        <v>6.6435495464912363E-3</v>
+      </c>
+      <c r="N53" s="3">
+        <f t="shared" si="2"/>
+        <v>23.916778367368451</v>
       </c>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
@@ -3612,26 +3609,26 @@
       <c r="G54" s="3">
         <v>200</v>
       </c>
-      <c r="H54" s="6">
+      <c r="H54" s="5">
         <v>220</v>
       </c>
-      <c r="I54" s="6"/>
+      <c r="I54" s="5"/>
       <c r="J54" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K54" s="4">
-        <f t="shared" si="2"/>
+      <c r="K54" s="3">
+        <f t="shared" si="1"/>
         <v>3.8013271108436497E-2</v>
       </c>
-      <c r="L54" s="6">
+      <c r="L54" s="5">
         <v>0.9</v>
       </c>
-      <c r="M54" s="4">
-        <f>L54*K54</f>
+      <c r="M54" s="3">
+        <f t="shared" si="3"/>
         <v>3.421194399759285E-2</v>
       </c>
-      <c r="N54" s="4">
-        <f t="shared" si="0"/>
+      <c r="N54" s="3">
+        <f t="shared" si="2"/>
         <v>123.16299839133426</v>
       </c>
     </row>
@@ -3651,26 +3648,26 @@
       <c r="G55" s="3">
         <v>80</v>
       </c>
-      <c r="H55" s="6">
+      <c r="H55" s="5">
         <v>88.9</v>
       </c>
-      <c r="I55" s="6">
+      <c r="I55" s="5">
         <v>4</v>
       </c>
       <c r="J55" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K55" s="4">
-        <f t="shared" si="2"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L55" s="6"/>
-      <c r="M55" s="4">
-        <f>L55*K55</f>
-        <v>0</v>
-      </c>
-      <c r="N55" s="4">
-        <f t="shared" si="0"/>
+      <c r="K55" s="3">
+        <f t="shared" si="1"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L55" s="5"/>
+      <c r="M55" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N55" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3696,26 +3693,26 @@
       <c r="G56" s="3">
         <v>100</v>
       </c>
-      <c r="H56" s="6">
+      <c r="H56" s="5">
         <v>114</v>
       </c>
-      <c r="I56" s="6">
+      <c r="I56" s="5">
         <v>4.5</v>
       </c>
       <c r="J56" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K56" s="4">
-        <f t="shared" si="2"/>
-        <v>9.4171203286762539E-3</v>
-      </c>
-      <c r="L56" s="6"/>
-      <c r="M56" s="4">
-        <f>L56*K56</f>
-        <v>0</v>
-      </c>
-      <c r="N56" s="4">
-        <f t="shared" si="0"/>
+      <c r="K56" s="3">
+        <f t="shared" si="1"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="L56" s="5"/>
+      <c r="M56" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N56" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3741,27 +3738,29 @@
       <c r="G57" s="3">
         <v>65</v>
       </c>
-      <c r="H57" s="6">
+      <c r="H57" s="5">
         <v>76.099999999999994</v>
       </c>
-      <c r="I57" s="6">
+      <c r="I57" s="5">
         <v>3.6</v>
       </c>
       <c r="J57" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K57" s="4">
-        <f t="shared" si="2"/>
-        <v>4.1282490963578371E-3</v>
-      </c>
-      <c r="L57" s="6"/>
-      <c r="M57" s="4">
-        <f>L57*K57</f>
-        <v>0</v>
-      </c>
-      <c r="N57" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="K57" s="3">
+        <f>PI()*(((H57-2*I57)*10^-3)^2/4)</f>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L57" s="5">
+        <v>1.1000000000000001</v>
+      </c>
+      <c r="M57" s="3">
+        <f t="shared" si="3"/>
+        <v>4.1012950167881989E-3</v>
+      </c>
+      <c r="N57" s="3">
+        <f t="shared" si="2"/>
+        <v>14.764662060437516</v>
       </c>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
@@ -3786,27 +3785,29 @@
       <c r="G58" s="3">
         <v>65</v>
       </c>
-      <c r="H58" s="6">
+      <c r="H58" s="5">
         <v>76.099999999999994</v>
       </c>
-      <c r="I58" s="6">
+      <c r="I58" s="5">
         <v>3.6</v>
       </c>
       <c r="J58" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K58" s="4">
-        <f t="shared" si="2"/>
-        <v>4.1282490963578371E-3</v>
-      </c>
-      <c r="L58" s="6"/>
-      <c r="M58" s="4">
-        <f>L58*K58</f>
-        <v>0</v>
-      </c>
-      <c r="N58" s="4">
-        <f t="shared" si="0"/>
-        <v>0</v>
+      <c r="K58" s="3">
+        <f t="shared" si="1"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L58" s="5">
+        <v>1</v>
+      </c>
+      <c r="M58" s="3">
+        <f t="shared" si="3"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="N58" s="3">
+        <f t="shared" si="2"/>
+        <v>13.422420054943197</v>
       </c>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
@@ -3831,26 +3832,26 @@
       <c r="G59" s="3">
         <v>65</v>
       </c>
-      <c r="H59" s="6">
+      <c r="H59" s="5">
         <v>76.099999999999994</v>
       </c>
-      <c r="I59" s="6">
+      <c r="I59" s="5">
         <v>3.6</v>
       </c>
       <c r="J59" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K59" s="4">
-        <f t="shared" si="2"/>
-        <v>4.1282490963578371E-3</v>
-      </c>
-      <c r="L59" s="6"/>
-      <c r="M59" s="4">
-        <f>L59*K59</f>
-        <v>0</v>
-      </c>
-      <c r="N59" s="4">
-        <f t="shared" si="0"/>
+      <c r="K59" s="3">
+        <f t="shared" si="1"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L59" s="5"/>
+      <c r="M59" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N59" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3876,26 +3877,26 @@
       <c r="G60" s="3">
         <v>50</v>
       </c>
-      <c r="H60" s="6">
+      <c r="H60" s="5">
         <v>60.3</v>
       </c>
-      <c r="I60" s="6">
+      <c r="I60" s="5">
         <v>3.6</v>
       </c>
       <c r="J60" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K60" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L60" s="6"/>
-      <c r="M60" s="4">
-        <f>L60*K60</f>
-        <v>0</v>
-      </c>
-      <c r="N60" s="4">
-        <f t="shared" si="0"/>
+      <c r="K60" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L60" s="5"/>
+      <c r="M60" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N60" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3921,26 +3922,26 @@
       <c r="G61" s="3">
         <v>50</v>
       </c>
-      <c r="H61" s="6">
+      <c r="H61" s="5">
         <v>60.3</v>
       </c>
-      <c r="I61" s="6">
+      <c r="I61" s="5">
         <v>3.6</v>
       </c>
       <c r="J61" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K61" s="4">
-        <f t="shared" si="2"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L61" s="6"/>
-      <c r="M61" s="4">
-        <f>L61*K61</f>
-        <v>0</v>
-      </c>
-      <c r="N61" s="4">
-        <f t="shared" si="0"/>
+      <c r="K61" s="3">
+        <f t="shared" si="1"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L61" s="5"/>
+      <c r="M61" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N61" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -3966,26 +3967,26 @@
       <c r="G62" s="3">
         <v>32</v>
       </c>
-      <c r="H62" s="6">
+      <c r="H62" s="5">
         <v>42.2</v>
       </c>
-      <c r="I62" s="6">
+      <c r="I62" s="5">
         <v>3.2</v>
       </c>
       <c r="J62" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="K62" s="4">
-        <f t="shared" si="2"/>
-        <v>1.1945906065275189E-3</v>
-      </c>
-      <c r="L62" s="6"/>
-      <c r="M62" s="4">
-        <f>L62*K62</f>
-        <v>0</v>
-      </c>
-      <c r="N62" s="4">
-        <f t="shared" si="0"/>
+      <c r="K62" s="3">
+        <f t="shared" si="1"/>
+        <v>1.0065977021367059E-3</v>
+      </c>
+      <c r="L62" s="5"/>
+      <c r="M62" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N62" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4007,26 +4008,26 @@
       <c r="G63" s="3">
         <v>100</v>
       </c>
-      <c r="H63" s="6">
+      <c r="H63" s="5">
         <v>114</v>
       </c>
-      <c r="I63" s="6">
+      <c r="I63" s="5">
         <v>5</v>
       </c>
       <c r="J63" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K63" s="4">
-        <f t="shared" si="2"/>
-        <v>9.3313155793250824E-3</v>
-      </c>
-      <c r="L63" s="6"/>
-      <c r="M63" s="4">
-        <f>L63*K63</f>
-        <v>0</v>
-      </c>
-      <c r="N63" s="4">
-        <f t="shared" si="0"/>
+      <c r="K63" s="3">
+        <f t="shared" si="1"/>
+        <v>8.4948665353068026E-3</v>
+      </c>
+      <c r="L63" s="5"/>
+      <c r="M63" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N63" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4052,26 +4053,26 @@
       <c r="G64" s="3">
         <v>150</v>
       </c>
-      <c r="H64" s="6">
+      <c r="H64" s="5">
         <v>168.3</v>
       </c>
-      <c r="I64" s="6">
+      <c r="I64" s="5">
         <v>5</v>
       </c>
       <c r="J64" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K64" s="4">
-        <f t="shared" si="2"/>
-        <v>2.0944126429521787E-2</v>
-      </c>
-      <c r="L64" s="6"/>
-      <c r="M64" s="4">
-        <f>L64*K64</f>
-        <v>0</v>
-      </c>
-      <c r="N64" s="4">
-        <f t="shared" si="0"/>
+      <c r="K64" s="3">
+        <f t="shared" si="1"/>
+        <v>1.9681206182778688E-2</v>
+      </c>
+      <c r="L64" s="5"/>
+      <c r="M64" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N64" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4093,26 +4094,26 @@
       <c r="G65" s="3">
         <v>100</v>
       </c>
-      <c r="H65" s="6">
+      <c r="H65" s="5">
         <v>114</v>
       </c>
-      <c r="I65" s="6">
+      <c r="I65" s="5">
         <v>4.5</v>
       </c>
       <c r="J65" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K65" s="4">
-        <f t="shared" si="2"/>
-        <v>9.4171203286762539E-3</v>
-      </c>
-      <c r="L65" s="6"/>
-      <c r="M65" s="4">
-        <f>L65*K65</f>
-        <v>0</v>
-      </c>
-      <c r="N65" s="4">
-        <f t="shared" si="0"/>
+      <c r="K65" s="3">
+        <f t="shared" si="1"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="L65" s="5"/>
+      <c r="M65" s="3">
+        <f t="shared" si="3"/>
+        <v>0</v>
+      </c>
+      <c r="N65" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4138,26 +4139,26 @@
       <c r="G66" s="3">
         <v>65</v>
       </c>
-      <c r="H66" s="6">
+      <c r="H66" s="5">
         <v>73</v>
       </c>
-      <c r="I66" s="6">
+      <c r="I66" s="5">
         <v>3.6</v>
       </c>
       <c r="J66" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K66" s="4">
-        <f t="shared" ref="K66:K71" si="3">PI()*(((H66-I66)*10^-3)^2/4)</f>
-        <v>3.7827602982609342E-3</v>
-      </c>
-      <c r="L66" s="6"/>
-      <c r="M66" s="4">
-        <f>L66*K66</f>
-        <v>0</v>
-      </c>
-      <c r="N66" s="4">
-        <f t="shared" si="0"/>
+      <c r="K66" s="3">
+        <f t="shared" si="1"/>
+        <v>3.4004913041721279E-3</v>
+      </c>
+      <c r="L66" s="5"/>
+      <c r="M66" s="3">
+        <f t="shared" ref="M66:M97" si="4">L66*K66</f>
+        <v>0</v>
+      </c>
+      <c r="N66" s="3">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
@@ -4183,26 +4184,26 @@
       <c r="G67" s="3">
         <v>65</v>
       </c>
-      <c r="H67" s="6">
+      <c r="H67" s="5">
         <v>76.099999999999994</v>
       </c>
-      <c r="I67" s="6">
+      <c r="I67" s="5">
         <v>3.6</v>
       </c>
       <c r="J67" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K67" s="4">
-        <f t="shared" si="3"/>
-        <v>4.1282490963578371E-3</v>
-      </c>
-      <c r="L67" s="6"/>
-      <c r="M67" s="4">
-        <f>L67*K67</f>
-        <v>0</v>
-      </c>
-      <c r="N67" s="4">
-        <f t="shared" ref="N67:N71" si="4">M67*3600</f>
+      <c r="K67" s="3">
+        <f t="shared" ref="K67:K71" si="5">PI()*(((H67-2*I67)*10^-3)^2/4)</f>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L67" s="5"/>
+      <c r="M67" s="3">
+        <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="N67" s="3">
+        <f t="shared" ref="N67:N71" si="6">M67*3600</f>
         <v>0</v>
       </c>
     </row>
@@ -4224,26 +4225,26 @@
       <c r="G68" s="3">
         <v>50</v>
       </c>
-      <c r="H68" s="6">
+      <c r="H68" s="5">
         <v>60.3</v>
       </c>
-      <c r="I68" s="6">
+      <c r="I68" s="5">
         <v>3.6</v>
       </c>
       <c r="J68" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K68" s="4">
-        <f t="shared" si="3"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L68" s="6"/>
-      <c r="M68" s="4">
-        <f>L68*K68</f>
-        <v>0</v>
-      </c>
-      <c r="N68" s="4">
+      <c r="K68" s="3">
+        <f t="shared" si="5"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L68" s="5"/>
+      <c r="M68" s="3">
         <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="N68" s="3">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -4265,26 +4266,26 @@
       <c r="G69" s="3">
         <v>50</v>
       </c>
-      <c r="H69" s="6">
+      <c r="H69" s="5">
         <v>60.3</v>
       </c>
-      <c r="I69" s="6">
+      <c r="I69" s="5">
         <v>3.6</v>
       </c>
       <c r="J69" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K69" s="4">
-        <f t="shared" si="3"/>
-        <v>2.524968701524822E-3</v>
-      </c>
-      <c r="L69" s="6"/>
-      <c r="M69" s="4">
-        <f>L69*K69</f>
-        <v>0</v>
-      </c>
-      <c r="N69" s="4">
+      <c r="K69" s="3">
+        <f t="shared" si="5"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L69" s="5"/>
+      <c r="M69" s="3">
         <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="N69" s="3">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -4304,26 +4305,26 @@
       <c r="G70" s="3">
         <v>100</v>
       </c>
-      <c r="H70" s="6">
+      <c r="H70" s="5">
         <v>114</v>
       </c>
-      <c r="I70" s="6">
+      <c r="I70" s="5">
         <v>4.5</v>
       </c>
       <c r="J70" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K70" s="4">
-        <f t="shared" si="3"/>
-        <v>9.4171203286762539E-3</v>
-      </c>
-      <c r="L70" s="6"/>
-      <c r="M70" s="4">
-        <f>L70*K70</f>
-        <v>0</v>
-      </c>
-      <c r="N70" s="4">
+      <c r="K70" s="3">
+        <f t="shared" si="5"/>
+        <v>8.6590147514568668E-3</v>
+      </c>
+      <c r="L70" s="5"/>
+      <c r="M70" s="3">
         <f t="shared" si="4"/>
+        <v>0</v>
+      </c>
+      <c r="N70" s="3">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
@@ -4343,31 +4344,30 @@
       <c r="G71" s="3">
         <v>80</v>
       </c>
-      <c r="H71" s="6">
+      <c r="H71" s="5">
         <v>88.9</v>
       </c>
-      <c r="I71" s="6">
+      <c r="I71" s="5">
         <v>4</v>
       </c>
       <c r="J71" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="K71" s="4">
-        <f t="shared" si="3"/>
-        <v>5.661157815750442E-3</v>
-      </c>
-      <c r="L71" s="6"/>
-      <c r="M71" s="4">
-        <f>L71*K71</f>
-        <v>0</v>
-      </c>
-      <c r="N71" s="4">
+      <c r="K71" s="3">
+        <f t="shared" si="5"/>
+        <v>5.1402817537852556E-3</v>
+      </c>
+      <c r="L71" s="5"/>
+      <c r="M71" s="3">
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
+      <c r="N71" s="3">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="g3d3e1Fm2tFm+4Kpa7Itvx8njHFV8W6HiKgvAfEhMHuCEZtGXwq24UkJFmJ6avfqAxiWLNS1MlfLLDfCwfaVWA==" saltValue="r+1d25qDUUEIwfXgXx7U7A==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <autoFilter ref="A1:N1" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:M72">
     <sortCondition ref="C40:C72"/>

</xml_diff>

<commit_message>
millora dels excels, edit colors sankey
</commit_message>
<xml_diff>
--- a/data/punts/punts-mesura-at.xlsx
+++ b/data/punts/punts-mesura-at.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\punts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EFDC6187-A128-43B5-BBC5-A1100F6C7CB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F49900FE-BD47-49D0-BA11-DD1DF48713C7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
@@ -4154,7 +4154,7 @@
       </c>
       <c r="L66" s="5"/>
       <c r="M66" s="3">
-        <f t="shared" ref="M66:M97" si="4">L66*K66</f>
+        <f t="shared" ref="M66:M71" si="4">L66*K66</f>
         <v>0</v>
       </c>
       <c r="N66" s="3">

</xml_diff>

<commit_message>
Simulador acabat, el dia que rebo el sensor!
</commit_message>
<xml_diff>
--- a/data/punts/punts-mesura-at.xlsx
+++ b/data/punts/punts-mesura-at.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ArnauCoronado\Documents_local\euromed\sxs\data\punts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7DFE0AA-45CC-4C77-944D-45B086AA12DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A1AB8AC-434F-424B-B264-AC4D13B79A69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{4CA701B3-5EB8-45D8-B6BB-1F057196BE44}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="362" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="396" uniqueCount="255">
   <si>
     <t>id</t>
   </si>
@@ -726,6 +726,84 @@
   </si>
   <si>
     <t>measured speed</t>
+  </si>
+  <si>
+    <t>GF-ASS</t>
+  </si>
+  <si>
+    <t>GF-ASS-1</t>
+  </si>
+  <si>
+    <t>GF-ASS-2</t>
+  </si>
+  <si>
+    <t>GF-ASS-3</t>
+  </si>
+  <si>
+    <t>GF-ASS-4</t>
+  </si>
+  <si>
+    <t>Y-190-1</t>
+  </si>
+  <si>
+    <t>Y-190-2</t>
+  </si>
+  <si>
+    <t>Y-180-3</t>
+  </si>
+  <si>
+    <t>Y-180-4</t>
+  </si>
+  <si>
+    <t>Nautas</t>
+  </si>
+  <si>
+    <t>SS-3000</t>
+  </si>
+  <si>
+    <t>SS-1000</t>
+  </si>
+  <si>
+    <t>S-600</t>
+  </si>
+  <si>
+    <t>SI-603</t>
+  </si>
+  <si>
+    <t>S-2100/S-2200</t>
+  </si>
+  <si>
+    <t>S-2100/S-2201</t>
+  </si>
+  <si>
+    <t>S-2100/S-2202</t>
+  </si>
+  <si>
+    <t>S-2100/S-2203</t>
+  </si>
+  <si>
+    <t>S-2100/S-2204</t>
+  </si>
+  <si>
+    <t>SI-2107</t>
+  </si>
+  <si>
+    <t>SI-2x07</t>
+  </si>
+  <si>
+    <t>SI-2207</t>
+  </si>
+  <si>
+    <t>SS-2100</t>
+  </si>
+  <si>
+    <t>SS-2200</t>
+  </si>
+  <si>
+    <t>S-6000</t>
+  </si>
+  <si>
+    <t>S-6002</t>
   </si>
 </sst>
 </file>
@@ -1170,13 +1248,13 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:O77"/>
+  <dimension ref="A1:O87"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="8.88671875" style="1"/>
     <col min="3" max="3" width="13" style="1" customWidth="1"/>
     <col min="4" max="4" width="15.6640625" style="1" customWidth="1"/>
-    <col min="5" max="5" width="13.77734375" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.88671875" style="1" customWidth="1"/>
     <col min="6" max="6" width="10.5546875" style="1" customWidth="1"/>
     <col min="7" max="7" width="5.44140625" style="1" customWidth="1"/>
     <col min="8" max="8" width="9.5546875" style="6" customWidth="1"/>
@@ -4433,7 +4511,7 @@
         <v>84</v>
       </c>
       <c r="K66" s="3">
-        <f t="shared" ref="K66:K71" si="6">PI()*(((H66-2*I66)*10^-3)^2/4)</f>
+        <f t="shared" ref="K66:K87" si="6">PI()*(((H66-2*I66)*10^-3)^2/4)</f>
         <v>8.4948665353068026E-3</v>
       </c>
       <c r="L66" s="5"/>
@@ -4697,105 +4775,620 @@
     </row>
     <row r="72" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A72" s="3">
-        <v>0</v>
+        <v>0.08</v>
       </c>
       <c r="B72" s="3">
-        <v>0</v>
-      </c>
-      <c r="C72" s="3"/>
-      <c r="D72" s="3"/>
-      <c r="E72" s="3"/>
+        <v>0.32800000000000001</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="E72" s="3" t="s">
+        <v>234</v>
+      </c>
       <c r="F72" s="3"/>
-      <c r="G72" s="3"/>
-      <c r="H72" s="3"/>
-      <c r="I72" s="3"/>
-      <c r="J72" s="3"/>
-      <c r="K72" s="3"/>
+      <c r="G72" s="3">
+        <v>65</v>
+      </c>
+      <c r="H72" s="3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="I72" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J72" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K72" s="3">
+        <f t="shared" si="6"/>
+        <v>3.728450015261999E-3</v>
+      </c>
       <c r="L72" s="3"/>
-      <c r="M72" s="3"/>
-      <c r="N72" s="3"/>
-      <c r="O72" s="3"/>
+      <c r="M72" s="3">
+        <v>1</v>
+      </c>
+      <c r="N72" s="3">
+        <f t="shared" ref="N72:N86" si="10">M72*K72</f>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="O72" s="3">
+        <f t="shared" ref="O72:O75" si="11">N72*3600</f>
+        <v>13.422420054943197</v>
+      </c>
     </row>
     <row r="73" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A73" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="B73" s="3">
+        <v>0.34100000000000003</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="E73" s="3" t="s">
+        <v>235</v>
+      </c>
+      <c r="F73" s="3"/>
+      <c r="G73" s="3">
+        <v>65</v>
+      </c>
+      <c r="H73" s="3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="I73" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J73" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K73" s="3">
+        <f t="shared" si="6"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L73" s="3"/>
+      <c r="M73" s="3">
+        <v>1</v>
+      </c>
+      <c r="N73" s="3">
+        <f t="shared" si="10"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="O73" s="3">
+        <f t="shared" si="11"/>
+        <v>13.422420054943197</v>
+      </c>
+    </row>
+    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A74" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="B74" s="3">
+        <v>0.36799999999999999</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>232</v>
+      </c>
+      <c r="E74" s="3" t="s">
+        <v>236</v>
+      </c>
+      <c r="F74" s="3"/>
+      <c r="G74" s="3">
+        <v>65</v>
+      </c>
+      <c r="H74" s="3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="I74" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J74" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K74" s="3">
+        <f t="shared" si="6"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L74" s="3"/>
+      <c r="M74" s="3">
+        <v>1</v>
+      </c>
+      <c r="N74" s="3">
+        <f t="shared" si="10"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="O74" s="3">
+        <f t="shared" si="11"/>
+        <v>13.422420054943197</v>
+      </c>
+    </row>
+    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A75" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="B75" s="3">
+        <v>0.374</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>233</v>
+      </c>
+      <c r="E75" s="3" t="s">
+        <v>237</v>
+      </c>
+      <c r="F75" s="3"/>
+      <c r="G75" s="3">
+        <v>65</v>
+      </c>
+      <c r="H75" s="3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="I75" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J75" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="K75" s="3">
+        <f t="shared" si="6"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L75" s="3"/>
+      <c r="M75" s="3">
+        <v>1</v>
+      </c>
+      <c r="N75" s="3">
+        <f t="shared" si="10"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="O75" s="3">
+        <f t="shared" si="11"/>
+        <v>13.422420054943197</v>
+      </c>
+    </row>
+    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A76" s="3"/>
+      <c r="B76" s="3"/>
+      <c r="C76" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E76" s="3" t="str">
+        <f>D76&amp;"01"</f>
+        <v>SS-300001</v>
+      </c>
+      <c r="F76" s="3"/>
+      <c r="G76" s="3">
+        <v>50</v>
+      </c>
+      <c r="H76" s="3">
+        <v>60.3</v>
+      </c>
+      <c r="I76" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J76" s="3"/>
+      <c r="K76" s="3">
+        <f t="shared" si="6"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L76" s="3"/>
+      <c r="M76" s="3">
+        <v>1</v>
+      </c>
+      <c r="N76" s="3">
+        <f t="shared" si="10"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="O76" s="3">
+        <f t="shared" ref="O76:O86" si="12">N76*3600</f>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A77" s="3">
+        <v>0.28199999999999997</v>
+      </c>
+      <c r="B77" s="3">
+        <v>0.33600000000000002</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>238</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>240</v>
+      </c>
+      <c r="E77" s="3" t="str">
+        <f>D77&amp;"02"</f>
+        <v>SS-100002</v>
+      </c>
+      <c r="F77" s="3"/>
+      <c r="G77" s="3">
+        <v>50</v>
+      </c>
+      <c r="H77" s="3">
+        <v>60.3</v>
+      </c>
+      <c r="I77" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J77" s="3"/>
+      <c r="K77" s="3">
+        <f t="shared" si="6"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L77" s="3"/>
+      <c r="M77" s="3">
+        <v>1</v>
+      </c>
+      <c r="N77" s="3">
+        <f t="shared" si="10"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="O77" s="3">
+        <f t="shared" si="12"/>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="78" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A78" s="3">
+        <v>0.16800000000000001</v>
+      </c>
+      <c r="B78" s="3">
+        <v>0.63700000000000001</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>241</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>242</v>
+      </c>
+      <c r="E78" s="3" t="str">
+        <f>D78&amp;1</f>
+        <v>SI-6031</v>
+      </c>
+      <c r="F78" s="3"/>
+      <c r="G78" s="3">
+        <v>65</v>
+      </c>
+      <c r="H78" s="3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="I78" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J78" s="3"/>
+      <c r="K78" s="3">
+        <f t="shared" si="6"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L78" s="3"/>
+      <c r="M78" s="3">
+        <v>1</v>
+      </c>
+      <c r="N78" s="3">
+        <f t="shared" si="10"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="O78" s="3">
+        <f t="shared" si="12"/>
+        <v>13.422420054943197</v>
+      </c>
+    </row>
+    <row r="79" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A79" s="3">
+        <v>6.3E-2</v>
+      </c>
+      <c r="B79" s="3">
+        <v>0.08</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>243</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>248</v>
+      </c>
+      <c r="E79" s="3" t="str">
+        <f>D79&amp;"01"</f>
+        <v>SI-210701</v>
+      </c>
+      <c r="F79" s="3"/>
+      <c r="G79" s="3">
+        <v>65</v>
+      </c>
+      <c r="H79" s="3">
+        <v>76.099999999999994</v>
+      </c>
+      <c r="I79" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J79" s="3"/>
+      <c r="K79" s="3">
+        <f t="shared" si="6"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="L79" s="3"/>
+      <c r="M79" s="3">
+        <v>1</v>
+      </c>
+      <c r="N79" s="3">
+        <f t="shared" si="10"/>
+        <v>3.728450015261999E-3</v>
+      </c>
+      <c r="O79" s="3">
+        <f t="shared" si="12"/>
+        <v>13.422420054943197</v>
+      </c>
+    </row>
+    <row r="80" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A80" s="3">
+        <v>7.5999999999999998E-2</v>
+      </c>
+      <c r="B80" s="3">
+        <v>0.84099999999999997</v>
+      </c>
+      <c r="C80" s="3" t="s">
+        <v>244</v>
+      </c>
+      <c r="D80" s="3" t="s">
+        <v>250</v>
+      </c>
+      <c r="E80" s="3" t="str">
+        <f>D80&amp;"02"</f>
+        <v>SI-220702</v>
+      </c>
+      <c r="F80" s="3"/>
+      <c r="G80" s="3">
+        <v>50</v>
+      </c>
+      <c r="H80" s="3">
+        <v>60.3</v>
+      </c>
+      <c r="I80" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J80" s="3"/>
+      <c r="K80" s="3">
+        <f t="shared" si="6"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L80" s="3"/>
+      <c r="M80" s="3">
+        <v>1</v>
+      </c>
+      <c r="N80" s="3">
+        <f t="shared" si="10"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="O80" s="3">
+        <f t="shared" si="12"/>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="81" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A81" s="3">
+        <v>8.2000000000000003E-2</v>
+      </c>
+      <c r="B81" s="3">
+        <v>0.86799999999999999</v>
+      </c>
+      <c r="C81" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="D81" s="3" t="s">
+        <v>249</v>
+      </c>
+      <c r="E81" s="3" t="str">
+        <f>D81&amp;"03"</f>
+        <v>SI-2x0703</v>
+      </c>
+      <c r="F81" s="3"/>
+      <c r="G81" s="3">
+        <v>80</v>
+      </c>
+      <c r="H81" s="3">
+        <v>88.9</v>
+      </c>
+      <c r="I81" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J81" s="3"/>
+      <c r="K81" s="3">
+        <f t="shared" si="6"/>
+        <v>5.2424463468799948E-3</v>
+      </c>
+      <c r="L81" s="3"/>
+      <c r="M81" s="3">
+        <v>1</v>
+      </c>
+      <c r="N81" s="3">
+        <f t="shared" si="10"/>
+        <v>5.2424463468799948E-3</v>
+      </c>
+      <c r="O81" s="3">
+        <f t="shared" si="12"/>
+        <v>18.872806848767983</v>
+      </c>
+    </row>
+    <row r="82" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A82" s="3"/>
+      <c r="B82" s="3"/>
+      <c r="C82" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="D82" s="3" t="s">
+        <v>251</v>
+      </c>
+      <c r="E82" s="3" t="str">
+        <f>D82&amp;"04"</f>
+        <v>SS-210004</v>
+      </c>
+      <c r="F82" s="3"/>
+      <c r="G82" s="3">
+        <v>50</v>
+      </c>
+      <c r="H82" s="3">
+        <v>60.3</v>
+      </c>
+      <c r="I82" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J82" s="3"/>
+      <c r="K82" s="3">
+        <f t="shared" si="6"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L82" s="3"/>
+      <c r="M82" s="3">
+        <v>1</v>
+      </c>
+      <c r="N82" s="3">
+        <f t="shared" si="10"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="O82" s="3">
+        <f t="shared" si="12"/>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="83" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A83" s="3"/>
+      <c r="B83" s="3"/>
+      <c r="C83" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="D83" s="3" t="s">
+        <v>252</v>
+      </c>
+      <c r="E83" s="3" t="str">
+        <f>D83&amp;"05"</f>
+        <v>SS-220005</v>
+      </c>
+      <c r="F83" s="3"/>
+      <c r="G83" s="3">
+        <v>50</v>
+      </c>
+      <c r="H83" s="3">
+        <v>60.3</v>
+      </c>
+      <c r="I83" s="3">
+        <v>3.6</v>
+      </c>
+      <c r="J83" s="3"/>
+      <c r="K83" s="3">
+        <f t="shared" si="6"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="L83" s="3"/>
+      <c r="M83" s="3">
+        <v>1</v>
+      </c>
+      <c r="N83" s="3">
+        <f t="shared" si="10"/>
+        <v>2.2145165154970788E-3</v>
+      </c>
+      <c r="O83" s="3">
+        <f t="shared" si="12"/>
+        <v>7.9722594557894837</v>
+      </c>
+    </row>
+    <row r="84" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="A84" s="3">
+        <v>0.10199999999999999</v>
+      </c>
+      <c r="B84" s="3">
+        <v>0.86299999999999999</v>
+      </c>
+      <c r="C84" s="3" t="s">
+        <v>253</v>
+      </c>
+      <c r="D84" s="3" t="s">
+        <v>254</v>
+      </c>
+      <c r="E84" s="3" t="str">
+        <f>D84&amp;1</f>
+        <v>S-60021</v>
+      </c>
+      <c r="F84" s="3"/>
+      <c r="G84" s="3">
+        <v>100</v>
+      </c>
+      <c r="H84" s="3">
+        <v>114.3</v>
+      </c>
+      <c r="I84" s="3">
+        <v>5</v>
+      </c>
+      <c r="J84" s="3"/>
+      <c r="K84" s="3">
+        <f t="shared" si="6"/>
+        <v>8.5439460665375083E-3</v>
+      </c>
+      <c r="L84" s="3"/>
+      <c r="M84" s="3">
+        <v>1</v>
+      </c>
+      <c r="N84" s="3">
+        <f t="shared" si="10"/>
+        <v>8.5439460665375083E-3</v>
+      </c>
+      <c r="O84" s="3">
+        <f t="shared" si="12"/>
+        <v>30.75820583953503</v>
+      </c>
+    </row>
+    <row r="85" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K85" s="3">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="B73" s="3">
+      <c r="M85" s="3">
+        <v>1</v>
+      </c>
+      <c r="N85" s="3">
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="C73" s="3"/>
-      <c r="D73" s="3"/>
-      <c r="E73" s="3"/>
-      <c r="F73" s="3"/>
-      <c r="G73" s="3"/>
-      <c r="H73" s="3"/>
-      <c r="I73" s="3"/>
-      <c r="J73" s="3"/>
-      <c r="K73" s="3"/>
-      <c r="L73" s="3"/>
-      <c r="M73" s="3"/>
-      <c r="N73" s="3"/>
-      <c r="O73" s="3"/>
-    </row>
-    <row r="74" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C74" s="3"/>
-      <c r="D74" s="3"/>
-      <c r="E74" s="3"/>
-      <c r="F74" s="3"/>
-      <c r="G74" s="3"/>
-      <c r="H74" s="3"/>
-      <c r="I74" s="3"/>
-      <c r="J74" s="3"/>
-      <c r="K74" s="3"/>
-      <c r="L74" s="3"/>
-      <c r="M74" s="3"/>
-      <c r="N74" s="3"/>
-      <c r="O74" s="3"/>
-    </row>
-    <row r="75" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C75" s="3"/>
-      <c r="D75" s="3"/>
-      <c r="E75" s="3"/>
-      <c r="F75" s="3"/>
-      <c r="G75" s="3"/>
-      <c r="H75" s="3"/>
-      <c r="I75" s="3"/>
-      <c r="J75" s="3"/>
-      <c r="K75" s="3"/>
-      <c r="L75" s="3"/>
-      <c r="M75" s="3"/>
-      <c r="N75" s="3"/>
-      <c r="O75" s="3"/>
-    </row>
-    <row r="76" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C76" s="3"/>
-      <c r="D76" s="3"/>
-      <c r="E76" s="3"/>
-      <c r="F76" s="3"/>
-      <c r="G76" s="3"/>
-      <c r="H76" s="3"/>
-      <c r="I76" s="3"/>
-      <c r="J76" s="3"/>
-      <c r="K76" s="3"/>
-      <c r="L76" s="3"/>
-      <c r="M76" s="3"/>
-      <c r="N76" s="3"/>
-      <c r="O76" s="3"/>
-    </row>
-    <row r="77" spans="1:15" x14ac:dyDescent="0.3">
-      <c r="C77" s="3"/>
-      <c r="D77" s="3"/>
-      <c r="E77" s="3"/>
-      <c r="F77" s="3"/>
-      <c r="G77" s="3"/>
-      <c r="H77" s="3"/>
-      <c r="I77" s="3"/>
-      <c r="J77" s="3"/>
-      <c r="K77" s="3"/>
-      <c r="L77" s="3"/>
-      <c r="M77" s="3"/>
-      <c r="N77" s="3"/>
-      <c r="O77" s="3"/>
+      <c r="O85" s="3">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="86" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K86" s="3">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="M86" s="3">
+        <v>1</v>
+      </c>
+      <c r="N86" s="3">
+        <f t="shared" si="10"/>
+        <v>0</v>
+      </c>
+      <c r="O86" s="3">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="87" spans="1:15" x14ac:dyDescent="0.3">
+      <c r="K87" s="3">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O1" xr:uid="{80D9219E-119C-467C-9531-507D24E0A5C1}">

</xml_diff>